<commit_message>
Atualização automática (27/10/2026 10:30): data/planilha_2026_cache.xlsx, data/planilha_cache.xlsx, data/pca_2027_cache.xlsx, data/contratacoes_2026_cache.xlsx
</commit_message>
<xml_diff>
--- a/data/contratacoes_2026_cache.xlsx
+++ b/data/contratacoes_2026_cache.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://goiasgovbr-my.sharepoint.com/personal/kelly_alexandria_goias_gov_br/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BAA9E7F7-EADD-46E5-816C-0D5B0ACBC517}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8CA54B82-CE5D-48F6-8F7A-66B35BA002B6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28740" windowHeight="9870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Contratações 2026" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_FilterDatabase" localSheetId="0" hidden="1">'Contratações 2026'!$A$1:$K$44</definedName>
+    <definedName name="_FilterDatabase" localSheetId="0" hidden="1">'Contratações 2026'!$A$1:$K$45</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="417" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="164">
   <si>
     <t>Prioridade</t>
   </si>
@@ -89,45 +89,51 @@
     <t>Materiais gráficos e brindes personalizados.</t>
   </si>
   <si>
+    <t>Julgamento da proposta. Apreciando documentos dos lotes III e IV. Demais aprovados.</t>
+  </si>
+  <si>
+    <t>Parte do orçamento deve ser gasto em 2026</t>
+  </si>
+  <si>
+    <t>Já possui</t>
+  </si>
+  <si>
+    <t>Sim</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pádua </t>
+  </si>
+  <si>
+    <t>SGI</t>
+  </si>
+  <si>
+    <t>118323</t>
+  </si>
+  <si>
+    <t>202600005000736</t>
+  </si>
+  <si>
+    <t>Mão de Obra - Motorista</t>
+  </si>
+  <si>
+    <t>Julgamento da proposta. Sessão será retomada dia 27/10 às 14h</t>
+  </si>
+  <si>
+    <t>Contrato atual vence dia 31/12/2026</t>
+  </si>
+  <si>
+    <t>107924</t>
+  </si>
+  <si>
+    <t>202400005027258</t>
+  </si>
+  <si>
+    <t>OCR MÓVEL</t>
+  </si>
+  <si>
     <t>Julgamento da proposta</t>
   </si>
   <si>
-    <t>Parte do orçamento deve ser gasto em 2026</t>
-  </si>
-  <si>
-    <t>Já possui</t>
-  </si>
-  <si>
-    <t>Sim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Pádua </t>
-  </si>
-  <si>
-    <t>SGI</t>
-  </si>
-  <si>
-    <t>118323</t>
-  </si>
-  <si>
-    <t>202600005000736</t>
-  </si>
-  <si>
-    <t>Mão de Obra - Motorista</t>
-  </si>
-  <si>
-    <t>Contrato atual vence dia 31/12/2026</t>
-  </si>
-  <si>
-    <t>107924</t>
-  </si>
-  <si>
-    <t>202400005027258</t>
-  </si>
-  <si>
-    <t>OCR MÓVEL</t>
-  </si>
-  <si>
     <t>Sem contrato</t>
   </si>
   <si>
@@ -146,7 +152,7 @@
     <t>Top System</t>
   </si>
   <si>
-    <t>Autorização do Ordenador</t>
+    <t>Aguardando empenho</t>
   </si>
   <si>
     <t>Contrato vence em 02/11/26</t>
@@ -161,39 +167,42 @@
     <t>Aquisição de Computadores (Workstation)</t>
   </si>
   <si>
+    <t>No jurídico para emissão de Parecer Prévio desde 26/10</t>
+  </si>
+  <si>
+    <t>Despesa deve ser empenhada até dia 16/11</t>
+  </si>
+  <si>
+    <t>Mariana</t>
+  </si>
+  <si>
+    <t>STI</t>
+  </si>
+  <si>
+    <t>Telas Interativas</t>
+  </si>
+  <si>
+    <t>Equipe de Planejamento atendendo diligências do agente e GELC elaborando as minutas.</t>
+  </si>
+  <si>
+    <t>Prorrogação com Supressão</t>
+  </si>
+  <si>
+    <t>Link de Dados Móveis - Via Direta</t>
+  </si>
+  <si>
+    <t>Fase Preparatória</t>
+  </si>
+  <si>
+    <t>Vence dia 08/12/2026</t>
+  </si>
+  <si>
+    <t>Mão de obra Nível Superior</t>
+  </si>
+  <si>
     <t>No jurídico para emissão de Parecer Prévio</t>
   </si>
   <si>
-    <t>Despesa deve ser empenhada até dia 16/11</t>
-  </si>
-  <si>
-    <t>Mariana</t>
-  </si>
-  <si>
-    <t>STI</t>
-  </si>
-  <si>
-    <t>Telas Interativas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Equipe de Planejamento atendendo diligências do agente </t>
-  </si>
-  <si>
-    <t>Prorrogação com Supressão</t>
-  </si>
-  <si>
-    <t>Link de Dados Móveis - Via Direta</t>
-  </si>
-  <si>
-    <t>Fase Preparatória</t>
-  </si>
-  <si>
-    <t>Vence dia 08/12/2026</t>
-  </si>
-  <si>
-    <t>Mão de obra Nível Superior</t>
-  </si>
-  <si>
     <t>Vence dia 17/11/2026</t>
   </si>
   <si>
@@ -203,6 +212,9 @@
     <t>Vigilância Armada</t>
   </si>
   <si>
+    <t>Análise do Processo e elaboração de minutas desde 27/10</t>
+  </si>
+  <si>
     <t>Vence dia 01/12/2026</t>
   </si>
   <si>
@@ -227,6 +239,9 @@
     <t>Vence dia 28/12/2026. Será realizada supressão?</t>
   </si>
   <si>
+    <t>Prorrogação com Acréscimo</t>
+  </si>
+  <si>
     <t>Licenças Microsoft</t>
   </si>
   <si>
@@ -335,7 +350,7 @@
     <t>Ponto de Acesso modelo Sem Fio Wi-fi</t>
   </si>
   <si>
-    <t>Equipe de Planejamento atendendo diligência Cactic</t>
+    <t>Aguardando Autorização do Ordenador</t>
   </si>
   <si>
     <t>117705</t>
@@ -386,6 +401,9 @@
     <t>Plataforma de capacitação on-line Alura</t>
   </si>
   <si>
+    <t>Termo de Homologação e Empenho</t>
+  </si>
+  <si>
     <t>123430</t>
   </si>
   <si>
@@ -408,6 +426,9 @@
   </si>
   <si>
     <t>Locação de veículos - Titano</t>
+  </si>
+  <si>
+    <t>Materiais de expediente</t>
   </si>
   <si>
     <t>Locação de veículos - S10</t>
@@ -749,16 +770,16 @@
     <xf numFmtId="1" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1063,11 +1084,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:O52"/>
+  <dimension ref="A1:O53"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.140625" customWidth="1"/>
-    <col min="2" max="2" width="23.140625" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="23.140625" customWidth="1"/>
     <col min="3" max="3" width="24" customWidth="1"/>
     <col min="4" max="4" width="24" style="6" customWidth="1"/>
     <col min="5" max="5" width="45" customWidth="1"/>
@@ -1117,7 +1138,7 @@
       <c r="N1" s="35"/>
       <c r="O1" s="35"/>
     </row>
-    <row r="2" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
         <v>11</v>
       </c>
@@ -1173,10 +1194,10 @@
         <v>24</v>
       </c>
       <c r="F3" s="18" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="G3" s="20" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H3" s="11" t="s">
         <v>18</v>
@@ -1200,22 +1221,22 @@
         <v>11</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E4" s="18" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F4" s="18" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="G4" s="20" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H4" s="11" t="s">
         <v>18</v>
@@ -1224,10 +1245,10 @@
         <v>19</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="K4" s="21" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="L4" s="37"/>
       <c r="M4" s="37"/>
@@ -1239,22 +1260,22 @@
         <v>11</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E5" s="13" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>18</v>
@@ -1263,7 +1284,7 @@
         <v>19</v>
       </c>
       <c r="J5" s="15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K5" s="16" t="s">
         <v>21</v>
@@ -1281,19 +1302,19 @@
         <v>123335</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E6" s="13" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="G6" s="22" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>19</v>
@@ -1302,17 +1323,17 @@
         <v>19</v>
       </c>
       <c r="J6" s="15" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L6" s="38"/>
       <c r="M6" s="38"/>
       <c r="N6" s="38"/>
       <c r="O6" s="38"/>
     </row>
-    <row r="7" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
         <v>11</v>
       </c>
@@ -1326,13 +1347,13 @@
         <v>14</v>
       </c>
       <c r="E7" s="24" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="F7" s="18" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="G7" s="22" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H7" s="23" t="s">
         <v>19</v>
@@ -1344,7 +1365,7 @@
         <v>20</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L7" s="38"/>
       <c r="M7" s="38"/>
@@ -1360,16 +1381,16 @@
         <v>202500004075118</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E8" s="24" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F8" s="29" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G8" s="22" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H8" s="23" t="s">
         <v>19</v>
@@ -1379,7 +1400,7 @@
       </c>
       <c r="J8" s="15"/>
       <c r="K8" s="15" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="L8" s="38"/>
       <c r="M8" s="38"/>
@@ -1395,16 +1416,16 @@
         <v>202500005005125</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E9" s="24" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F9" s="29" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="G9" s="22" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H9" s="23" t="s">
         <v>19</v>
@@ -1413,7 +1434,7 @@
         <v>19</v>
       </c>
       <c r="J9" s="15" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="K9" s="15" t="s">
         <v>21</v>
@@ -1432,16 +1453,16 @@
         <v>202500005000718</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E10" s="24" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="F10" s="29" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G10" s="22" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H10" s="23" t="s">
         <v>19</v>
@@ -1467,16 +1488,16 @@
         <v>201700004040059</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="E11" s="24" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F11" s="29" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="G11" s="22" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H11" s="23" t="s">
         <v>19</v>
@@ -1502,16 +1523,16 @@
         <v>201700004044816</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E12" s="24" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F12" s="29" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="G12" s="22" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="H12" s="23" t="s">
         <v>19</v>
@@ -1528,7 +1549,7 @@
       <c r="N12" s="38"/>
       <c r="O12" s="38"/>
     </row>
-    <row r="13" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>11</v>
       </c>
@@ -1537,16 +1558,16 @@
         <v>202500005018321</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="E13" s="24" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="F13" s="29" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="G13" s="22" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="H13" s="23" t="s">
         <v>19</v>
@@ -1556,7 +1577,7 @@
       </c>
       <c r="J13" s="15"/>
       <c r="K13" s="15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L13" s="38"/>
       <c r="M13" s="38"/>
@@ -1567,7 +1588,7 @@
       <c r="A14" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="24">
+      <c r="B14" s="17">
         <v>122462</v>
       </c>
       <c r="C14" s="23">
@@ -1577,23 +1598,23 @@
         <v>14</v>
       </c>
       <c r="E14" s="24" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="F14" s="13" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="G14" s="22" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H14" s="23" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I14" s="23" t="s">
         <v>19</v>
       </c>
       <c r="J14" s="15"/>
       <c r="K14" s="15" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="L14" s="38"/>
       <c r="M14" s="38"/>
@@ -1604,29 +1625,29 @@
       <c r="A15" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="17">
         <v>118979</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D15" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E15" s="13" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="F15" s="13" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="G15" s="22" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="H15" s="11" t="s">
         <v>19</v>
       </c>
       <c r="I15" s="11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J15" s="15"/>
       <c r="K15" s="15" t="s">
@@ -1642,28 +1663,28 @@
         <v>11</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D16" s="20" t="s">
         <v>14</v>
       </c>
       <c r="E16" s="18" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="F16" s="18" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="G16" s="22" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="H16" s="17" t="s">
         <v>19</v>
       </c>
       <c r="I16" s="17" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="J16" s="15"/>
       <c r="K16" s="15" t="s">
@@ -1676,33 +1697,33 @@
     </row>
     <row r="17" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="9" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B17" s="17"/>
       <c r="C17" s="23">
         <v>202400004002472</v>
       </c>
       <c r="D17" s="12" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E17" s="24" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="F17" s="29" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="G17" s="22" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H17" s="23" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I17" s="23" t="s">
         <v>19</v>
       </c>
       <c r="J17" s="15"/>
       <c r="K17" s="15" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="L17" s="38"/>
       <c r="M17" s="38"/>
@@ -1711,33 +1732,33 @@
     </row>
     <row r="18" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B18" s="17"/>
       <c r="C18" s="23">
         <v>202300005025089</v>
       </c>
       <c r="D18" s="12" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="E18" s="24" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="F18" s="29" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="G18" s="22" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H18" s="23" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I18" s="23" t="s">
         <v>19</v>
       </c>
       <c r="J18" s="15"/>
       <c r="K18" s="15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L18" s="38"/>
       <c r="M18" s="38"/>
@@ -1746,23 +1767,23 @@
     </row>
     <row r="19" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="9" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B19" s="17"/>
       <c r="C19" s="23">
         <v>202400005007478</v>
       </c>
       <c r="D19" s="12" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E19" s="24" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="F19" s="29" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G19" s="22" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="H19" s="23" t="s">
         <v>19</v>
@@ -1772,7 +1793,7 @@
       </c>
       <c r="J19" s="15"/>
       <c r="K19" s="15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L19" s="38"/>
       <c r="M19" s="38"/>
@@ -1781,23 +1802,23 @@
     </row>
     <row r="20" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B20" s="17"/>
       <c r="C20" s="23">
         <v>202300004068367</v>
       </c>
       <c r="D20" s="12" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E20" s="24" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="F20" s="29" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G20" s="22" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="H20" s="23" t="s">
         <v>19</v>
@@ -1807,7 +1828,7 @@
       </c>
       <c r="J20" s="15"/>
       <c r="K20" s="15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L20" s="38"/>
       <c r="M20" s="38"/>
@@ -1816,23 +1837,23 @@
     </row>
     <row r="21" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B21" s="17"/>
       <c r="C21" s="23">
         <v>202300004068367</v>
       </c>
       <c r="D21" s="12" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E21" s="24" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="F21" s="29" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G21" s="22" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="H21" s="23" t="s">
         <v>19</v>
@@ -1842,7 +1863,7 @@
       </c>
       <c r="J21" s="15"/>
       <c r="K21" s="15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L21" s="38"/>
       <c r="M21" s="38"/>
@@ -1851,23 +1872,23 @@
     </row>
     <row r="22" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B22" s="17"/>
       <c r="C22" s="23">
         <v>202300004068367</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E22" s="24" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="F22" s="29" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G22" s="22" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="H22" s="23" t="s">
         <v>19</v>
@@ -1877,7 +1898,7 @@
       </c>
       <c r="J22" s="15"/>
       <c r="K22" s="15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L22" s="38"/>
       <c r="M22" s="38"/>
@@ -1886,23 +1907,23 @@
     </row>
     <row r="23" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B23" s="17"/>
       <c r="C23" s="23">
         <v>202300004068367</v>
       </c>
       <c r="D23" s="12" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E23" s="24" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="F23" s="29" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G23" s="22" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="H23" s="23" t="s">
         <v>19</v>
@@ -1912,7 +1933,7 @@
       </c>
       <c r="J23" s="15"/>
       <c r="K23" s="15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L23" s="38"/>
       <c r="M23" s="38"/>
@@ -1921,23 +1942,23 @@
     </row>
     <row r="24" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B24" s="17"/>
       <c r="C24" s="23">
         <v>202400005042407</v>
       </c>
       <c r="D24" s="12" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E24" s="24" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="F24" s="29" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="G24" s="22" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="H24" s="23" t="s">
         <v>19</v>
@@ -1956,23 +1977,23 @@
     </row>
     <row r="25" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B25" s="17"/>
       <c r="C25" s="23">
         <v>202400005005765</v>
       </c>
       <c r="D25" s="12" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E25" s="24" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="F25" s="29" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G25" s="22" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="H25" s="23" t="s">
         <v>19</v>
@@ -1991,23 +2012,23 @@
     </row>
     <row r="26" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B26" s="17"/>
       <c r="C26" s="23">
         <v>202400005005765</v>
       </c>
       <c r="D26" s="12" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E26" s="24" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="F26" s="29" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G26" s="22" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="H26" s="23" t="s">
         <v>19</v>
@@ -2024,27 +2045,27 @@
       <c r="N26" s="38"/>
       <c r="O26" s="38"/>
     </row>
-    <row r="27" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:15" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B27" s="17" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="C27" s="17" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="D27" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E27" s="18" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="F27" s="18" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="G27" s="22" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H27" s="17" t="s">
         <v>18</v>
@@ -2053,10 +2074,10 @@
         <v>19</v>
       </c>
       <c r="J27" s="15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K27" s="21" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L27" s="37"/>
       <c r="M27" s="37"/>
@@ -2065,25 +2086,25 @@
     </row>
     <row r="28" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="C28" s="17" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="D28" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="F28" s="18" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="G28" s="22" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H28" s="17" t="s">
         <v>18</v>
@@ -2092,7 +2113,7 @@
         <v>19</v>
       </c>
       <c r="J28" s="15" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="K28" s="21" t="s">
         <v>21</v>
@@ -2104,25 +2125,25 @@
     </row>
     <row r="29" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="D29" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="G29" s="12" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="H29" s="11" t="s">
         <v>19</v>
@@ -2131,7 +2152,7 @@
         <v>19</v>
       </c>
       <c r="J29" s="15" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="K29" s="16" t="s">
         <v>21</v>
@@ -2143,37 +2164,37 @@
     </row>
     <row r="30" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="D30" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E30" s="13" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="G30" s="22" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H30" s="11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I30" s="11" t="s">
         <v>19</v>
       </c>
       <c r="J30" s="15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K30" s="16" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L30" s="36"/>
       <c r="M30" s="36"/>
@@ -2182,37 +2203,37 @@
     </row>
     <row r="31" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="D31" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E31" s="26" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="F31" s="26" t="s">
-        <v>35</v>
+        <v>120</v>
       </c>
       <c r="G31" s="22" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H31" s="11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I31" s="11" t="s">
         <v>19</v>
       </c>
       <c r="J31" s="15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K31" s="16" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L31" s="36"/>
       <c r="M31" s="36"/>
@@ -2221,76 +2242,76 @@
     </row>
     <row r="32" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="9" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B32" s="17" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="C32" s="17" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="D32" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E32" s="18" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="F32" s="13" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="G32" s="22" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H32" s="17" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I32" s="17" t="s">
         <v>19</v>
       </c>
       <c r="J32" s="15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K32" s="21" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L32" s="37"/>
       <c r="M32" s="37"/>
       <c r="N32" s="37"/>
       <c r="O32" s="37"/>
     </row>
-    <row r="33" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:15" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="9" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="D33" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E33" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="F33" s="26" t="s">
-        <v>48</v>
+        <v>126</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>116</v>
       </c>
       <c r="G33" s="22" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H33" s="11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="I33" s="11" t="s">
         <v>19</v>
       </c>
       <c r="J33" s="15" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="K33" s="16" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L33" s="36"/>
       <c r="M33" s="36"/>
@@ -2299,23 +2320,23 @@
     </row>
     <row r="34" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="9" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="B34" s="11"/>
       <c r="C34" s="23">
         <v>202400005040749</v>
       </c>
       <c r="D34" s="12" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E34" s="13" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="F34" s="26" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G34" s="22" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="H34" s="23" t="s">
         <v>19</v>
@@ -2324,7 +2345,7 @@
         <v>19</v>
       </c>
       <c r="J34" s="15" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="K34" s="16" t="s">
         <v>21</v>
@@ -2335,35 +2356,29 @@
       <c r="O34" s="36"/>
     </row>
     <row r="35" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="9"/>
+      <c r="A35" s="9" t="s">
+        <v>88</v>
+      </c>
       <c r="B35" s="11"/>
-      <c r="C35" s="23">
-        <v>202400005040749</v>
-      </c>
+      <c r="C35" s="23"/>
       <c r="D35" s="12" t="s">
-        <v>80</v>
+        <v>14</v>
       </c>
       <c r="E35" s="13" t="s">
-        <v>123</v>
-      </c>
-      <c r="F35" s="26" t="s">
-        <v>48</v>
-      </c>
+        <v>129</v>
+      </c>
+      <c r="F35" s="26"/>
       <c r="G35" s="22" t="s">
-        <v>91</v>
+        <v>43</v>
       </c>
       <c r="H35" s="23" t="s">
-        <v>19</v>
+        <v>71</v>
       </c>
       <c r="I35" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="J35" s="15" t="s">
-        <v>52</v>
-      </c>
-      <c r="K35" s="16" t="s">
-        <v>21</v>
-      </c>
+      <c r="J35" s="15"/>
+      <c r="K35" s="16"/>
       <c r="L35" s="36"/>
       <c r="M35" s="36"/>
       <c r="N35" s="36"/>
@@ -2371,23 +2386,23 @@
     </row>
     <row r="36" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="9" t="s">
-        <v>73</v>
+        <v>88</v>
       </c>
       <c r="B36" s="11"/>
       <c r="C36" s="23">
         <v>202400005040749</v>
       </c>
       <c r="D36" s="12" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E36" s="13" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="F36" s="26" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G36" s="22" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="H36" s="23" t="s">
         <v>19</v>
@@ -2396,7 +2411,7 @@
         <v>19</v>
       </c>
       <c r="J36" s="15" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="K36" s="16" t="s">
         <v>21</v>
@@ -2408,23 +2423,23 @@
     </row>
     <row r="37" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="9" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B37" s="11"/>
       <c r="C37" s="23">
         <v>202400005040749</v>
       </c>
       <c r="D37" s="12" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="E37" s="13" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="F37" s="26" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="G37" s="22" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="H37" s="23" t="s">
         <v>19</v>
@@ -2433,7 +2448,7 @@
         <v>19</v>
       </c>
       <c r="J37" s="15" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="K37" s="16" t="s">
         <v>21</v>
@@ -2445,37 +2460,35 @@
     </row>
     <row r="38" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="B38" s="17">
-        <v>123535</v>
-      </c>
-      <c r="C38" s="17" t="s">
-        <v>126</v>
+        <v>78</v>
+      </c>
+      <c r="B38" s="11"/>
+      <c r="C38" s="23">
+        <v>202400005040749</v>
       </c>
       <c r="D38" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="E38" s="18" t="s">
-        <v>127</v>
-      </c>
-      <c r="F38" s="18" t="s">
-        <v>128</v>
+        <v>85</v>
+      </c>
+      <c r="E38" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="F38" s="26" t="s">
+        <v>50</v>
       </c>
       <c r="G38" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="H38" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="I38" s="17" t="s">
+        <v>96</v>
+      </c>
+      <c r="H38" s="23" t="s">
+        <v>19</v>
+      </c>
+      <c r="I38" s="23" t="s">
         <v>19</v>
       </c>
       <c r="J38" s="15" t="s">
-        <v>129</v>
+        <v>55</v>
       </c>
       <c r="K38" s="16" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="L38" s="36"/>
       <c r="M38" s="36"/>
@@ -2483,38 +2496,38 @@
       <c r="O38" s="36"/>
     </row>
     <row r="39" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="B39" s="11" t="s">
-        <v>131</v>
-      </c>
-      <c r="C39" s="11" t="s">
-        <v>132</v>
+      <c r="A39" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="B39" s="17">
+        <v>123535</v>
+      </c>
+      <c r="C39" s="17" t="s">
+        <v>133</v>
       </c>
       <c r="D39" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E39" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="F39" s="13" t="s">
-        <v>65</v>
-      </c>
-      <c r="G39" s="14" t="s">
-        <v>77</v>
-      </c>
-      <c r="H39" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="I39" s="11" t="s">
-        <v>66</v>
+      <c r="E39" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="F39" s="18" t="s">
+        <v>135</v>
+      </c>
+      <c r="G39" s="22" t="s">
+        <v>43</v>
+      </c>
+      <c r="H39" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="I39" s="17" t="s">
+        <v>19</v>
       </c>
       <c r="J39" s="15" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="K39" s="16" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="L39" s="36"/>
       <c r="M39" s="36"/>
@@ -2523,37 +2536,37 @@
     </row>
     <row r="40" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="B40" s="17" t="s">
-        <v>135</v>
-      </c>
-      <c r="C40" s="17" t="s">
-        <v>136</v>
+        <v>137</v>
+      </c>
+      <c r="B40" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="C40" s="11" t="s">
+        <v>139</v>
       </c>
       <c r="D40" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E40" s="18" t="s">
-        <v>137</v>
-      </c>
-      <c r="F40" s="18" t="s">
-        <v>65</v>
-      </c>
-      <c r="G40" s="19" t="s">
-        <v>138</v>
-      </c>
-      <c r="H40" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="I40" s="17" t="s">
-        <v>66</v>
+      <c r="E40" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="F40" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="G40" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="H40" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="I40" s="11" t="s">
+        <v>71</v>
       </c>
       <c r="J40" s="15" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="K40" s="16" t="s">
-        <v>21</v>
+        <v>33</v>
       </c>
       <c r="L40" s="36"/>
       <c r="M40" s="36"/>
@@ -2562,37 +2575,37 @@
     </row>
     <row r="41" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C41" s="17" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D41" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E41" s="18" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F41" s="18" t="s">
-        <v>143</v>
-      </c>
-      <c r="G41" s="20" t="s">
-        <v>144</v>
+        <v>70</v>
+      </c>
+      <c r="G41" s="19" t="s">
+        <v>145</v>
       </c>
       <c r="H41" s="17" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I41" s="17" t="s">
-        <v>19</v>
+        <v>71</v>
       </c>
       <c r="J41" s="15" t="s">
-        <v>52</v>
+        <v>146</v>
       </c>
       <c r="K41" s="16" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="L41" s="36"/>
       <c r="M41" s="36"/>
@@ -2601,37 +2614,37 @@
     </row>
     <row r="42" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="B42" s="11" t="s">
-        <v>145</v>
-      </c>
-      <c r="C42" s="11" t="s">
-        <v>146</v>
+        <v>137</v>
+      </c>
+      <c r="B42" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="C42" s="17" t="s">
+        <v>148</v>
       </c>
       <c r="D42" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E42" s="13" t="s">
-        <v>147</v>
-      </c>
-      <c r="F42" s="13" t="s">
-        <v>148</v>
-      </c>
-      <c r="G42" s="12" t="s">
+      <c r="E42" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="H42" s="11" t="s">
+      <c r="F42" s="18" t="s">
+        <v>150</v>
+      </c>
+      <c r="G42" s="20" t="s">
+        <v>151</v>
+      </c>
+      <c r="H42" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="I42" s="11" t="s">
+      <c r="I42" s="17" t="s">
         <v>19</v>
       </c>
       <c r="J42" s="15" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="K42" s="16" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="L42" s="36"/>
       <c r="M42" s="36"/>
@@ -2640,37 +2653,37 @@
     </row>
     <row r="43" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="B43" s="17" t="s">
-        <v>150</v>
-      </c>
-      <c r="C43" s="17" t="s">
-        <v>150</v>
+        <v>137</v>
+      </c>
+      <c r="B43" s="11" t="s">
+        <v>152</v>
+      </c>
+      <c r="C43" s="11" t="s">
+        <v>153</v>
       </c>
       <c r="D43" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="E43" s="18" t="s">
-        <v>151</v>
-      </c>
-      <c r="F43" s="18" t="s">
-        <v>152</v>
-      </c>
-      <c r="G43" s="20" t="s">
-        <v>77</v>
-      </c>
-      <c r="H43" s="17" t="s">
+      <c r="E43" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="F43" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="G43" s="12" t="s">
+        <v>156</v>
+      </c>
+      <c r="H43" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="I43" s="17" t="s">
+      <c r="I43" s="11" t="s">
         <v>19</v>
       </c>
       <c r="J43" s="15" t="s">
-        <v>129</v>
+        <v>32</v>
       </c>
       <c r="K43" s="16" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="L43" s="36"/>
       <c r="M43" s="36"/>
@@ -2679,93 +2692,132 @@
     </row>
     <row r="44" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>130</v>
-      </c>
-      <c r="B44" s="27"/>
-      <c r="C44" s="27">
-        <v>202400005034383</v>
-      </c>
-      <c r="D44" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="B44" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="C44" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="D44" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E44" s="18" t="s">
-        <v>153</v>
-      </c>
-      <c r="F44" s="26" t="s">
-        <v>48</v>
-      </c>
-      <c r="G44" s="15" t="s">
-        <v>154</v>
-      </c>
-      <c r="H44" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="I44" s="27" t="s">
-        <v>66</v>
+        <v>158</v>
+      </c>
+      <c r="F44" s="18" t="s">
+        <v>159</v>
+      </c>
+      <c r="G44" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="H44" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="I44" s="17" t="s">
+        <v>19</v>
       </c>
       <c r="J44" s="15" t="s">
-        <v>155</v>
+        <v>136</v>
       </c>
       <c r="K44" s="16" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="L44" s="36"/>
       <c r="M44" s="36"/>
       <c r="N44" s="36"/>
       <c r="O44" s="36"/>
     </row>
-    <row r="45" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="F45" s="30"/>
-      <c r="G45" s="5"/>
-      <c r="H45"/>
-      <c r="I45"/>
+    <row r="45" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="B45" s="27"/>
+      <c r="C45" s="27">
+        <v>202400005034383</v>
+      </c>
+      <c r="D45" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="E45" s="18" t="s">
+        <v>160</v>
+      </c>
+      <c r="F45" s="26" t="s">
+        <v>50</v>
+      </c>
+      <c r="G45" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="H45" s="27" t="s">
+        <v>19</v>
+      </c>
+      <c r="I45" s="27" t="s">
+        <v>71</v>
+      </c>
+      <c r="J45" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="K45" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="L45" s="36"/>
+      <c r="M45" s="36"/>
+      <c r="N45" s="36"/>
+      <c r="O45" s="36"/>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="C46" s="1"/>
-      <c r="H46" s="33"/>
-      <c r="I46" s="33"/>
+      <c r="F46" s="30"/>
+      <c r="G46" s="5"/>
+      <c r="H46"/>
+      <c r="I46"/>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="G47" s="28"/>
-      <c r="H47"/>
-      <c r="I47" s="28" t="s">
-        <v>156</v>
-      </c>
-      <c r="J47" s="28"/>
-      <c r="K47" s="28"/>
-      <c r="L47" s="28"/>
-      <c r="M47" s="28"/>
-      <c r="N47" s="28"/>
-      <c r="O47" s="28"/>
+      <c r="C47" s="1"/>
+      <c r="H47" s="33"/>
+      <c r="I47" s="33"/>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="F48" s="30"/>
-      <c r="G48" s="5"/>
+      <c r="G48" s="28"/>
       <c r="H48"/>
-      <c r="I48"/>
+      <c r="I48" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="J48" s="28"/>
+      <c r="K48" s="28"/>
+      <c r="L48" s="28"/>
+      <c r="M48" s="28"/>
+      <c r="N48" s="28"/>
+      <c r="O48" s="28"/>
     </row>
     <row r="49" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C49" s="1"/>
-      <c r="H49" s="33"/>
-      <c r="I49" s="33"/>
+      <c r="F49" s="30"/>
+      <c r="G49" s="5"/>
+      <c r="H49"/>
+      <c r="I49"/>
     </row>
     <row r="50" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="H50"/>
-      <c r="I50"/>
+      <c r="C50" s="1"/>
+      <c r="H50" s="33"/>
+      <c r="I50" s="33"/>
     </row>
     <row r="51" spans="3:9" x14ac:dyDescent="0.25">
       <c r="H51"/>
       <c r="I51"/>
     </row>
     <row r="52" spans="3:9" x14ac:dyDescent="0.25">
-      <c r="C52" s="2"/>
-      <c r="F52" s="32"/>
-      <c r="G52" s="7"/>
-      <c r="H52" s="34"/>
-      <c r="I52" s="34"/>
+      <c r="H52"/>
+      <c r="I52"/>
+    </row>
+    <row r="53" spans="3:9" x14ac:dyDescent="0.25">
+      <c r="C53" s="2"/>
+      <c r="F53" s="32"/>
+      <c r="G53" s="7"/>
+      <c r="H53" s="34"/>
+      <c r="I53" s="34"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K44" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:K45" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualização automática (27/10/2026 10:37): app.py, sync_github.py, data/planilha_2026_cache.xlsx, data/pca_2027_cache.xlsx, data/contratacoes_2026_cache.xlsx
</commit_message>
<xml_diff>
--- a/data/contratacoes_2026_cache.xlsx
+++ b/data/contratacoes_2026_cache.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://goiasgovbr-my.sharepoint.com/personal/kelly_alexandria_goias_gov_br/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8CA54B82-CE5D-48F6-8F7A-66B35BA002B6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1A75923-2901-4A79-A520-C5EE761E97FC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28740" windowHeight="9870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="424" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="164">
   <si>
     <t>Prioridade</t>
   </si>
@@ -2359,15 +2359,21 @@
       <c r="A35" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="B35" s="11"/>
-      <c r="C35" s="23"/>
+      <c r="B35" s="11">
+        <v>123022</v>
+      </c>
+      <c r="C35" s="23">
+        <v>202600005030907</v>
+      </c>
       <c r="D35" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E35" s="13" t="s">
         <v>129</v>
       </c>
-      <c r="F35" s="26"/>
+      <c r="F35" s="26" t="s">
+        <v>50</v>
+      </c>
       <c r="G35" s="22" t="s">
         <v>43</v>
       </c>
@@ -2378,7 +2384,9 @@
         <v>19</v>
       </c>
       <c r="J35" s="15"/>
-      <c r="K35" s="16"/>
+      <c r="K35" s="16" t="s">
+        <v>21</v>
+      </c>
       <c r="L35" s="36"/>
       <c r="M35" s="36"/>
       <c r="N35" s="36"/>

</xml_diff>

<commit_message>
Atualização automática (27/10/2026 10:39): data/pca_2027_cache.xlsx, data/contratacoes_2026_cache.xlsx
</commit_message>
<xml_diff>
--- a/data/contratacoes_2026_cache.xlsx
+++ b/data/contratacoes_2026_cache.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://goiasgovbr-my.sharepoint.com/personal/kelly_alexandria_goias_gov_br/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1A75923-2901-4A79-A520-C5EE761E97FC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{0ECB8681-9AAA-4F6D-84F9-FF196C141ECC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28740" windowHeight="9870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -446,9 +446,6 @@
     <t>GitLab Premium</t>
   </si>
   <si>
-    <t xml:space="preserve">Aguardando cadastro Fornecedor </t>
-  </si>
-  <si>
     <t>Kelly</t>
   </si>
   <si>
@@ -531,6 +528,9 @@
   </si>
   <si>
     <t>Data da Atualização: 26/10/2026</t>
+  </si>
+  <si>
+    <t>Aguardando Validação CACTIC</t>
   </si>
 </sst>
 </file>
@@ -2520,7 +2520,7 @@
         <v>134</v>
       </c>
       <c r="F39" s="18" t="s">
-        <v>135</v>
+        <v>163</v>
       </c>
       <c r="G39" s="22" t="s">
         <v>43</v>
@@ -2532,7 +2532,7 @@
         <v>19</v>
       </c>
       <c r="J39" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K39" s="16" t="s">
         <v>45</v>
@@ -2544,19 +2544,19 @@
     </row>
     <row r="40" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="B40" s="11" t="s">
         <v>137</v>
       </c>
-      <c r="B40" s="11" t="s">
+      <c r="C40" s="11" t="s">
         <v>138</v>
-      </c>
-      <c r="C40" s="11" t="s">
-        <v>139</v>
       </c>
       <c r="D40" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F40" s="13" t="s">
         <v>70</v>
@@ -2571,7 +2571,7 @@
         <v>71</v>
       </c>
       <c r="J40" s="15" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="K40" s="16" t="s">
         <v>33</v>
@@ -2583,25 +2583,25 @@
     </row>
     <row r="41" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B41" s="17" t="s">
+        <v>141</v>
+      </c>
+      <c r="C41" s="17" t="s">
         <v>142</v>
-      </c>
-      <c r="C41" s="17" t="s">
-        <v>143</v>
       </c>
       <c r="D41" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E41" s="18" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F41" s="18" t="s">
         <v>70</v>
       </c>
       <c r="G41" s="19" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H41" s="17" t="s">
         <v>19</v>
@@ -2610,7 +2610,7 @@
         <v>71</v>
       </c>
       <c r="J41" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K41" s="16" t="s">
         <v>21</v>
@@ -2622,25 +2622,25 @@
     </row>
     <row r="42" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B42" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="C42" s="17" t="s">
         <v>147</v>
-      </c>
-      <c r="C42" s="17" t="s">
-        <v>148</v>
       </c>
       <c r="D42" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E42" s="18" t="s">
+        <v>148</v>
+      </c>
+      <c r="F42" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="F42" s="18" t="s">
+      <c r="G42" s="20" t="s">
         <v>150</v>
-      </c>
-      <c r="G42" s="20" t="s">
-        <v>151</v>
       </c>
       <c r="H42" s="17" t="s">
         <v>18</v>
@@ -2661,25 +2661,25 @@
     </row>
     <row r="43" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B43" s="11" t="s">
+        <v>151</v>
+      </c>
+      <c r="C43" s="11" t="s">
         <v>152</v>
-      </c>
-      <c r="C43" s="11" t="s">
-        <v>153</v>
       </c>
       <c r="D43" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E43" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="F43" s="13" t="s">
         <v>154</v>
       </c>
-      <c r="F43" s="13" t="s">
+      <c r="G43" s="12" t="s">
         <v>155</v>
-      </c>
-      <c r="G43" s="12" t="s">
-        <v>156</v>
       </c>
       <c r="H43" s="11" t="s">
         <v>18</v>
@@ -2700,22 +2700,22 @@
     </row>
     <row r="44" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B44" s="17" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C44" s="17" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D44" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E44" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="F44" s="18" t="s">
         <v>158</v>
-      </c>
-      <c r="F44" s="18" t="s">
-        <v>159</v>
       </c>
       <c r="G44" s="20" t="s">
         <v>82</v>
@@ -2727,7 +2727,7 @@
         <v>19</v>
       </c>
       <c r="J44" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K44" s="16" t="s">
         <v>33</v>
@@ -2739,7 +2739,7 @@
     </row>
     <row r="45" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="B45" s="27"/>
       <c r="C45" s="27">
@@ -2749,13 +2749,13 @@
         <v>14</v>
       </c>
       <c r="E45" s="18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F45" s="26" t="s">
         <v>50</v>
       </c>
       <c r="G45" s="15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H45" s="27" t="s">
         <v>19</v>
@@ -2764,7 +2764,7 @@
         <v>71</v>
       </c>
       <c r="J45" s="15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K45" s="16" t="s">
         <v>33</v>
@@ -2789,7 +2789,7 @@
       <c r="G48" s="28"/>
       <c r="H48"/>
       <c r="I48" s="28" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J48" s="28"/>
       <c r="K48" s="28"/>

</xml_diff>

<commit_message>
Atualização automática (27/10/2026 12:41): data/pca_2027_cache.xlsx, data/contratacoes_2026_cache.xlsx
</commit_message>
<xml_diff>
--- a/data/contratacoes_2026_cache.xlsx
+++ b/data/contratacoes_2026_cache.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://goiasgovbr-my.sharepoint.com/personal/kelly_alexandria_goias_gov_br/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{26B78D98-1BF1-4648-915B-3241D800A7E7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8EC7C637-33B1-44FD-BD4B-FA4F6A61E37C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28740" windowHeight="9870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -446,6 +446,9 @@
     <t>GitLab Premium</t>
   </si>
   <si>
+    <t xml:space="preserve">Aguardando cadastro Fornecedor </t>
+  </si>
+  <si>
     <t>Kelly</t>
   </si>
   <si>
@@ -528,9 +531,6 @@
   </si>
   <si>
     <t>Data da Atualização: 26/10/2026</t>
-  </si>
-  <si>
-    <t>Aguardando Validação CACTIC</t>
   </si>
 </sst>
 </file>
@@ -2520,7 +2520,7 @@
         <v>134</v>
       </c>
       <c r="F39" s="18" t="s">
-        <v>163</v>
+        <v>135</v>
       </c>
       <c r="G39" s="22" t="s">
         <v>43</v>
@@ -2532,7 +2532,7 @@
         <v>19</v>
       </c>
       <c r="J39" s="15" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K39" s="16" t="s">
         <v>45</v>
@@ -2544,19 +2544,19 @@
     </row>
     <row r="40" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C40" s="11" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D40" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E40" s="13" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F40" s="13" t="s">
         <v>70</v>
@@ -2571,7 +2571,7 @@
         <v>71</v>
       </c>
       <c r="J40" s="15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K40" s="16" t="s">
         <v>33</v>
@@ -2583,25 +2583,25 @@
     </row>
     <row r="41" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B41" s="17" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C41" s="17" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D41" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E41" s="18" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F41" s="18" t="s">
         <v>70</v>
       </c>
       <c r="G41" s="19" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H41" s="17" t="s">
         <v>19</v>
@@ -2610,7 +2610,7 @@
         <v>71</v>
       </c>
       <c r="J41" s="15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="K41" s="16" t="s">
         <v>21</v>
@@ -2622,25 +2622,25 @@
     </row>
     <row r="42" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B42" s="17" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C42" s="17" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D42" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E42" s="18" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F42" s="18" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G42" s="20" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H42" s="17" t="s">
         <v>18</v>
@@ -2661,25 +2661,25 @@
     </row>
     <row r="43" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C43" s="11" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D43" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E43" s="13" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F43" s="13" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G43" s="12" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H43" s="11" t="s">
         <v>18</v>
@@ -2700,22 +2700,22 @@
     </row>
     <row r="44" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B44" s="17" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C44" s="17" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D44" s="12" t="s">
         <v>14</v>
       </c>
       <c r="E44" s="18" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F44" s="18" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G44" s="20" t="s">
         <v>82</v>
@@ -2727,7 +2727,7 @@
         <v>19</v>
       </c>
       <c r="J44" s="15" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K44" s="16" t="s">
         <v>33</v>
@@ -2739,7 +2739,7 @@
     </row>
     <row r="45" spans="1:15" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B45" s="27"/>
       <c r="C45" s="27">
@@ -2749,13 +2749,13 @@
         <v>14</v>
       </c>
       <c r="E45" s="18" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F45" s="26" t="s">
         <v>50</v>
       </c>
       <c r="G45" s="15" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H45" s="27" t="s">
         <v>19</v>
@@ -2764,7 +2764,7 @@
         <v>71</v>
       </c>
       <c r="J45" s="15" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K45" s="16" t="s">
         <v>33</v>
@@ -2789,7 +2789,7 @@
       <c r="G48" s="28"/>
       <c r="H48"/>
       <c r="I48" s="28" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="J48" s="28"/>
       <c r="K48" s="28"/>

</xml_diff>